<commit_message>
Split vehicle maintenance costs into 유류비/정비비/기타 categories
일일기록 now has a 지출구분 dropdown (유류비/정비비/기타) plus
지출내용/지출금액, instead of one combined maintenance field, so
월별손익 and 연도별수익률 show fuel cost, repair cost, and other
costs as separate P&L line items instead of one lumped total.

Updates monthly_summary.py to match the new column layout and break
out the same three categories in the generated reconciliation message.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015A54uauDNpDF2TgGKkujty
</commit_message>
<xml_diff>
--- a/data/vehicle/5톤계란운송_손익관리.xlsx
+++ b/data/vehicle/5톤계란운송_손익관리.xlsx
@@ -14,7 +14,7 @@
     <sheet name="사용안내" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'일일기록'!$A$1:$I$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'일일기록'!$A$1:$J$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -271,6 +271,11 @@
     <comment ref="E1" authorId="0" shapeId="0">
       <text>
         <t>자동 계산: 판수 × 단가</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>지출 항목이 있는 행에만 유류비/정비비/기타 중 선택</t>
       </text>
     </comment>
   </commentList>
@@ -670,7 +675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -678,10 +683,11 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -712,20 +718,25 @@
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>차량유지내용</t>
+          <t>지출구분</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>차량유지비용</t>
+          <t>지출내용</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
+          <t>지출금액</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
           <t>하이패스</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>비고</t>
         </is>
@@ -754,11 +765,12 @@
         <v/>
       </c>
       <c r="F2" s="7" t="n"/>
-      <c r="G2" s="8" t="n"/>
-      <c r="H2" s="8" t="n">
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="8" t="n"/>
+      <c r="I2" s="8" t="n">
         <v>800000</v>
       </c>
-      <c r="I2" s="7" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>하이패스 월 충전</t>
         </is>
@@ -788,14 +800,19 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
+          <t>유류비</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
           <t>유류</t>
         </is>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="H3" s="8" t="n">
         <v>200000</v>
       </c>
-      <c r="H3" s="8" t="n"/>
-      <c r="I3" s="7" t="inlineStr">
+      <c r="I3" s="8" t="n"/>
+      <c r="J3" s="7" t="inlineStr">
         <is>
           <t>예시 행 - 실제 입력 시 삭제/수정</t>
         </is>
@@ -804,12 +821,12 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>2026-01-02</t>
+          <t>2026-01-03</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>상문</t>
+          <t>천금</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
@@ -823,15 +840,30 @@
         <f>IF(C4="","",C4*D4)</f>
         <v/>
       </c>
-      <c r="F4" s="7" t="n"/>
-      <c r="G4" s="8" t="n"/>
-      <c r="H4" s="8" t="n"/>
-      <c r="I4" s="7" t="inlineStr"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>정비비</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>엔진오일교환</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="n">
+        <v>294000</v>
+      </c>
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="n"/>
-      <c r="B5" s="11" t="n"/>
-      <c r="C5" s="12" t="n"/>
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="8" t="n"/>
       <c r="D5" s="9">
         <f>IF(C5="","",고정비설정!$B$3)</f>
         <v/>
@@ -840,15 +872,36 @@
         <f>IF(C5="","",C5*D5)</f>
         <v/>
       </c>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="12" t="n"/>
-      <c r="I5" s="11" t="n"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>기타</t>
+        </is>
+      </c>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>세차</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="n">
+        <v>30000</v>
+      </c>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="n"/>
-      <c r="B6" s="11" t="n"/>
-      <c r="C6" s="12" t="n"/>
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>상문</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>5040</v>
+      </c>
       <c r="D6" s="9">
         <f>IF(C6="","",고정비설정!$B$3)</f>
         <v/>
@@ -857,10 +910,11 @@
         <f>IF(C6="","",C6*D6)</f>
         <v/>
       </c>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="12" t="n"/>
-      <c r="I6" s="11" t="n"/>
+      <c r="F6" s="7" t="n"/>
+      <c r="G6" s="7" t="n"/>
+      <c r="H6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="7" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n"/>
@@ -875,9 +929,10 @@
         <v/>
       </c>
       <c r="F7" s="11" t="n"/>
-      <c r="G7" s="12" t="n"/>
+      <c r="G7" s="11" t="n"/>
       <c r="H7" s="12" t="n"/>
-      <c r="I7" s="11" t="n"/>
+      <c r="I7" s="12" t="n"/>
+      <c r="J7" s="11" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="n"/>
@@ -892,9 +947,10 @@
         <v/>
       </c>
       <c r="F8" s="11" t="n"/>
-      <c r="G8" s="12" t="n"/>
+      <c r="G8" s="11" t="n"/>
       <c r="H8" s="12" t="n"/>
-      <c r="I8" s="11" t="n"/>
+      <c r="I8" s="12" t="n"/>
+      <c r="J8" s="11" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="n"/>
@@ -909,9 +965,10 @@
         <v/>
       </c>
       <c r="F9" s="11" t="n"/>
-      <c r="G9" s="12" t="n"/>
+      <c r="G9" s="11" t="n"/>
       <c r="H9" s="12" t="n"/>
-      <c r="I9" s="11" t="n"/>
+      <c r="I9" s="12" t="n"/>
+      <c r="J9" s="11" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="n"/>
@@ -926,9 +983,10 @@
         <v/>
       </c>
       <c r="F10" s="11" t="n"/>
-      <c r="G10" s="12" t="n"/>
+      <c r="G10" s="11" t="n"/>
       <c r="H10" s="12" t="n"/>
-      <c r="I10" s="11" t="n"/>
+      <c r="I10" s="12" t="n"/>
+      <c r="J10" s="11" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>
@@ -943,9 +1001,10 @@
         <v/>
       </c>
       <c r="F11" s="11" t="n"/>
-      <c r="G11" s="12" t="n"/>
+      <c r="G11" s="11" t="n"/>
       <c r="H11" s="12" t="n"/>
-      <c r="I11" s="11" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="n"/>
@@ -960,9 +1019,10 @@
         <v/>
       </c>
       <c r="F12" s="11" t="n"/>
-      <c r="G12" s="12" t="n"/>
+      <c r="G12" s="11" t="n"/>
       <c r="H12" s="12" t="n"/>
-      <c r="I12" s="11" t="n"/>
+      <c r="I12" s="12" t="n"/>
+      <c r="J12" s="11" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="n"/>
@@ -977,9 +1037,10 @@
         <v/>
       </c>
       <c r="F13" s="11" t="n"/>
-      <c r="G13" s="12" t="n"/>
+      <c r="G13" s="11" t="n"/>
       <c r="H13" s="12" t="n"/>
-      <c r="I13" s="11" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="11" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="n"/>
@@ -994,9 +1055,10 @@
         <v/>
       </c>
       <c r="F14" s="11" t="n"/>
-      <c r="G14" s="12" t="n"/>
+      <c r="G14" s="11" t="n"/>
       <c r="H14" s="12" t="n"/>
-      <c r="I14" s="11" t="n"/>
+      <c r="I14" s="12" t="n"/>
+      <c r="J14" s="11" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="n"/>
@@ -1011,9 +1073,10 @@
         <v/>
       </c>
       <c r="F15" s="11" t="n"/>
-      <c r="G15" s="12" t="n"/>
+      <c r="G15" s="11" t="n"/>
       <c r="H15" s="12" t="n"/>
-      <c r="I15" s="11" t="n"/>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n"/>
@@ -1028,9 +1091,10 @@
         <v/>
       </c>
       <c r="F16" s="11" t="n"/>
-      <c r="G16" s="12" t="n"/>
+      <c r="G16" s="11" t="n"/>
       <c r="H16" s="12" t="n"/>
-      <c r="I16" s="11" t="n"/>
+      <c r="I16" s="12" t="n"/>
+      <c r="J16" s="11" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="n"/>
@@ -1045,9 +1109,10 @@
         <v/>
       </c>
       <c r="F17" s="11" t="n"/>
-      <c r="G17" s="12" t="n"/>
+      <c r="G17" s="11" t="n"/>
       <c r="H17" s="12" t="n"/>
-      <c r="I17" s="11" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="11" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="n"/>
@@ -1062,9 +1127,10 @@
         <v/>
       </c>
       <c r="F18" s="11" t="n"/>
-      <c r="G18" s="12" t="n"/>
+      <c r="G18" s="11" t="n"/>
       <c r="H18" s="12" t="n"/>
-      <c r="I18" s="11" t="n"/>
+      <c r="I18" s="12" t="n"/>
+      <c r="J18" s="11" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="n"/>
@@ -1079,9 +1145,10 @@
         <v/>
       </c>
       <c r="F19" s="11" t="n"/>
-      <c r="G19" s="12" t="n"/>
+      <c r="G19" s="11" t="n"/>
       <c r="H19" s="12" t="n"/>
-      <c r="I19" s="11" t="n"/>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="11" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="n"/>
@@ -1096,9 +1163,10 @@
         <v/>
       </c>
       <c r="F20" s="11" t="n"/>
-      <c r="G20" s="12" t="n"/>
+      <c r="G20" s="11" t="n"/>
       <c r="H20" s="12" t="n"/>
-      <c r="I20" s="11" t="n"/>
+      <c r="I20" s="12" t="n"/>
+      <c r="J20" s="11" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="n"/>
@@ -1113,9 +1181,10 @@
         <v/>
       </c>
       <c r="F21" s="11" t="n"/>
-      <c r="G21" s="12" t="n"/>
+      <c r="G21" s="11" t="n"/>
       <c r="H21" s="12" t="n"/>
-      <c r="I21" s="11" t="n"/>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="11" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="n"/>
@@ -1130,9 +1199,10 @@
         <v/>
       </c>
       <c r="F22" s="11" t="n"/>
-      <c r="G22" s="12" t="n"/>
+      <c r="G22" s="11" t="n"/>
       <c r="H22" s="12" t="n"/>
-      <c r="I22" s="11" t="n"/>
+      <c r="I22" s="12" t="n"/>
+      <c r="J22" s="11" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n"/>
@@ -1147,9 +1217,10 @@
         <v/>
       </c>
       <c r="F23" s="11" t="n"/>
-      <c r="G23" s="12" t="n"/>
+      <c r="G23" s="11" t="n"/>
       <c r="H23" s="12" t="n"/>
-      <c r="I23" s="11" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="11" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="n"/>
@@ -1164,9 +1235,10 @@
         <v/>
       </c>
       <c r="F24" s="11" t="n"/>
-      <c r="G24" s="12" t="n"/>
+      <c r="G24" s="11" t="n"/>
       <c r="H24" s="12" t="n"/>
-      <c r="I24" s="11" t="n"/>
+      <c r="I24" s="12" t="n"/>
+      <c r="J24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="n"/>
@@ -1181,9 +1253,10 @@
         <v/>
       </c>
       <c r="F25" s="11" t="n"/>
-      <c r="G25" s="12" t="n"/>
+      <c r="G25" s="11" t="n"/>
       <c r="H25" s="12" t="n"/>
-      <c r="I25" s="11" t="n"/>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="n"/>
@@ -1198,9 +1271,10 @@
         <v/>
       </c>
       <c r="F26" s="11" t="n"/>
-      <c r="G26" s="12" t="n"/>
+      <c r="G26" s="11" t="n"/>
       <c r="H26" s="12" t="n"/>
-      <c r="I26" s="11" t="n"/>
+      <c r="I26" s="12" t="n"/>
+      <c r="J26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="n"/>
@@ -1215,9 +1289,10 @@
         <v/>
       </c>
       <c r="F27" s="11" t="n"/>
-      <c r="G27" s="12" t="n"/>
+      <c r="G27" s="11" t="n"/>
       <c r="H27" s="12" t="n"/>
-      <c r="I27" s="11" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="11" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="n"/>
@@ -1232,9 +1307,10 @@
         <v/>
       </c>
       <c r="F28" s="11" t="n"/>
-      <c r="G28" s="12" t="n"/>
+      <c r="G28" s="11" t="n"/>
       <c r="H28" s="12" t="n"/>
-      <c r="I28" s="11" t="n"/>
+      <c r="I28" s="12" t="n"/>
+      <c r="J28" s="11" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="n"/>
@@ -1249,9 +1325,10 @@
         <v/>
       </c>
       <c r="F29" s="11" t="n"/>
-      <c r="G29" s="12" t="n"/>
+      <c r="G29" s="11" t="n"/>
       <c r="H29" s="12" t="n"/>
-      <c r="I29" s="11" t="n"/>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="n"/>
@@ -1266,9 +1343,10 @@
         <v/>
       </c>
       <c r="F30" s="11" t="n"/>
-      <c r="G30" s="12" t="n"/>
+      <c r="G30" s="11" t="n"/>
       <c r="H30" s="12" t="n"/>
-      <c r="I30" s="11" t="n"/>
+      <c r="I30" s="12" t="n"/>
+      <c r="J30" s="11" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="n"/>
@@ -1283,9 +1361,10 @@
         <v/>
       </c>
       <c r="F31" s="11" t="n"/>
-      <c r="G31" s="12" t="n"/>
+      <c r="G31" s="11" t="n"/>
       <c r="H31" s="12" t="n"/>
-      <c r="I31" s="11" t="n"/>
+      <c r="I31" s="12" t="n"/>
+      <c r="J31" s="11" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="n"/>
@@ -1300,9 +1379,10 @@
         <v/>
       </c>
       <c r="F32" s="11" t="n"/>
-      <c r="G32" s="12" t="n"/>
+      <c r="G32" s="11" t="n"/>
       <c r="H32" s="12" t="n"/>
-      <c r="I32" s="11" t="n"/>
+      <c r="I32" s="12" t="n"/>
+      <c r="J32" s="11" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="n"/>
@@ -1317,9 +1397,10 @@
         <v/>
       </c>
       <c r="F33" s="11" t="n"/>
-      <c r="G33" s="12" t="n"/>
+      <c r="G33" s="11" t="n"/>
       <c r="H33" s="12" t="n"/>
-      <c r="I33" s="11" t="n"/>
+      <c r="I33" s="12" t="n"/>
+      <c r="J33" s="11" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="n"/>
@@ -1334,9 +1415,10 @@
         <v/>
       </c>
       <c r="F34" s="11" t="n"/>
-      <c r="G34" s="12" t="n"/>
+      <c r="G34" s="11" t="n"/>
       <c r="H34" s="12" t="n"/>
-      <c r="I34" s="11" t="n"/>
+      <c r="I34" s="12" t="n"/>
+      <c r="J34" s="11" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="n"/>
@@ -1351,9 +1433,10 @@
         <v/>
       </c>
       <c r="F35" s="11" t="n"/>
-      <c r="G35" s="12" t="n"/>
+      <c r="G35" s="11" t="n"/>
       <c r="H35" s="12" t="n"/>
-      <c r="I35" s="11" t="n"/>
+      <c r="I35" s="12" t="n"/>
+      <c r="J35" s="11" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="n"/>
@@ -1368,9 +1451,10 @@
         <v/>
       </c>
       <c r="F36" s="11" t="n"/>
-      <c r="G36" s="12" t="n"/>
+      <c r="G36" s="11" t="n"/>
       <c r="H36" s="12" t="n"/>
-      <c r="I36" s="11" t="n"/>
+      <c r="I36" s="12" t="n"/>
+      <c r="J36" s="11" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n"/>
@@ -1385,9 +1469,10 @@
         <v/>
       </c>
       <c r="F37" s="11" t="n"/>
-      <c r="G37" s="12" t="n"/>
+      <c r="G37" s="11" t="n"/>
       <c r="H37" s="12" t="n"/>
-      <c r="I37" s="11" t="n"/>
+      <c r="I37" s="12" t="n"/>
+      <c r="J37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="n"/>
@@ -1402,9 +1487,10 @@
         <v/>
       </c>
       <c r="F38" s="11" t="n"/>
-      <c r="G38" s="12" t="n"/>
+      <c r="G38" s="11" t="n"/>
       <c r="H38" s="12" t="n"/>
-      <c r="I38" s="11" t="n"/>
+      <c r="I38" s="12" t="n"/>
+      <c r="J38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="n"/>
@@ -1419,9 +1505,10 @@
         <v/>
       </c>
       <c r="F39" s="11" t="n"/>
-      <c r="G39" s="12" t="n"/>
+      <c r="G39" s="11" t="n"/>
       <c r="H39" s="12" t="n"/>
-      <c r="I39" s="11" t="n"/>
+      <c r="I39" s="12" t="n"/>
+      <c r="J39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="n"/>
@@ -1436,9 +1523,10 @@
         <v/>
       </c>
       <c r="F40" s="11" t="n"/>
-      <c r="G40" s="12" t="n"/>
+      <c r="G40" s="11" t="n"/>
       <c r="H40" s="12" t="n"/>
-      <c r="I40" s="11" t="n"/>
+      <c r="I40" s="12" t="n"/>
+      <c r="J40" s="11" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="n"/>
@@ -1453,9 +1541,10 @@
         <v/>
       </c>
       <c r="F41" s="11" t="n"/>
-      <c r="G41" s="12" t="n"/>
+      <c r="G41" s="11" t="n"/>
       <c r="H41" s="12" t="n"/>
-      <c r="I41" s="11" t="n"/>
+      <c r="I41" s="12" t="n"/>
+      <c r="J41" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="n"/>
@@ -1470,9 +1559,10 @@
         <v/>
       </c>
       <c r="F42" s="11" t="n"/>
-      <c r="G42" s="12" t="n"/>
+      <c r="G42" s="11" t="n"/>
       <c r="H42" s="12" t="n"/>
-      <c r="I42" s="11" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="11" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="n"/>
@@ -1487,9 +1577,10 @@
         <v/>
       </c>
       <c r="F43" s="11" t="n"/>
-      <c r="G43" s="12" t="n"/>
+      <c r="G43" s="11" t="n"/>
       <c r="H43" s="12" t="n"/>
-      <c r="I43" s="11" t="n"/>
+      <c r="I43" s="12" t="n"/>
+      <c r="J43" s="11" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="n"/>
@@ -1504,9 +1595,10 @@
         <v/>
       </c>
       <c r="F44" s="11" t="n"/>
-      <c r="G44" s="12" t="n"/>
+      <c r="G44" s="11" t="n"/>
       <c r="H44" s="12" t="n"/>
-      <c r="I44" s="11" t="n"/>
+      <c r="I44" s="12" t="n"/>
+      <c r="J44" s="11" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n"/>
@@ -1521,9 +1613,10 @@
         <v/>
       </c>
       <c r="F45" s="11" t="n"/>
-      <c r="G45" s="12" t="n"/>
+      <c r="G45" s="11" t="n"/>
       <c r="H45" s="12" t="n"/>
-      <c r="I45" s="11" t="n"/>
+      <c r="I45" s="12" t="n"/>
+      <c r="J45" s="11" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="n"/>
@@ -1538,9 +1631,10 @@
         <v/>
       </c>
       <c r="F46" s="11" t="n"/>
-      <c r="G46" s="12" t="n"/>
+      <c r="G46" s="11" t="n"/>
       <c r="H46" s="12" t="n"/>
-      <c r="I46" s="11" t="n"/>
+      <c r="I46" s="12" t="n"/>
+      <c r="J46" s="11" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="n"/>
@@ -1555,9 +1649,10 @@
         <v/>
       </c>
       <c r="F47" s="11" t="n"/>
-      <c r="G47" s="12" t="n"/>
+      <c r="G47" s="11" t="n"/>
       <c r="H47" s="12" t="n"/>
-      <c r="I47" s="11" t="n"/>
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="11" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="n"/>
@@ -1572,9 +1667,10 @@
         <v/>
       </c>
       <c r="F48" s="11" t="n"/>
-      <c r="G48" s="12" t="n"/>
+      <c r="G48" s="11" t="n"/>
       <c r="H48" s="12" t="n"/>
-      <c r="I48" s="11" t="n"/>
+      <c r="I48" s="12" t="n"/>
+      <c r="J48" s="11" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="n"/>
@@ -1589,9 +1685,10 @@
         <v/>
       </c>
       <c r="F49" s="11" t="n"/>
-      <c r="G49" s="12" t="n"/>
+      <c r="G49" s="11" t="n"/>
       <c r="H49" s="12" t="n"/>
-      <c r="I49" s="11" t="n"/>
+      <c r="I49" s="12" t="n"/>
+      <c r="J49" s="11" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="n"/>
@@ -1606,9 +1703,10 @@
         <v/>
       </c>
       <c r="F50" s="11" t="n"/>
-      <c r="G50" s="12" t="n"/>
+      <c r="G50" s="11" t="n"/>
       <c r="H50" s="12" t="n"/>
-      <c r="I50" s="11" t="n"/>
+      <c r="I50" s="12" t="n"/>
+      <c r="J50" s="11" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="n"/>
@@ -1623,9 +1721,10 @@
         <v/>
       </c>
       <c r="F51" s="11" t="n"/>
-      <c r="G51" s="12" t="n"/>
+      <c r="G51" s="11" t="n"/>
       <c r="H51" s="12" t="n"/>
-      <c r="I51" s="11" t="n"/>
+      <c r="I51" s="12" t="n"/>
+      <c r="J51" s="11" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="n"/>
@@ -1640,9 +1739,10 @@
         <v/>
       </c>
       <c r="F52" s="11" t="n"/>
-      <c r="G52" s="12" t="n"/>
+      <c r="G52" s="11" t="n"/>
       <c r="H52" s="12" t="n"/>
-      <c r="I52" s="11" t="n"/>
+      <c r="I52" s="12" t="n"/>
+      <c r="J52" s="11" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="n"/>
@@ -1657,9 +1757,10 @@
         <v/>
       </c>
       <c r="F53" s="11" t="n"/>
-      <c r="G53" s="12" t="n"/>
+      <c r="G53" s="11" t="n"/>
       <c r="H53" s="12" t="n"/>
-      <c r="I53" s="11" t="n"/>
+      <c r="I53" s="12" t="n"/>
+      <c r="J53" s="11" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="n"/>
@@ -1674,9 +1775,10 @@
         <v/>
       </c>
       <c r="F54" s="11" t="n"/>
-      <c r="G54" s="12" t="n"/>
+      <c r="G54" s="11" t="n"/>
       <c r="H54" s="12" t="n"/>
-      <c r="I54" s="11" t="n"/>
+      <c r="I54" s="12" t="n"/>
+      <c r="J54" s="11" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="n"/>
@@ -1691,9 +1793,10 @@
         <v/>
       </c>
       <c r="F55" s="11" t="n"/>
-      <c r="G55" s="12" t="n"/>
+      <c r="G55" s="11" t="n"/>
       <c r="H55" s="12" t="n"/>
-      <c r="I55" s="11" t="n"/>
+      <c r="I55" s="12" t="n"/>
+      <c r="J55" s="11" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="n"/>
@@ -1708,9 +1811,10 @@
         <v/>
       </c>
       <c r="F56" s="11" t="n"/>
-      <c r="G56" s="12" t="n"/>
+      <c r="G56" s="11" t="n"/>
       <c r="H56" s="12" t="n"/>
-      <c r="I56" s="11" t="n"/>
+      <c r="I56" s="12" t="n"/>
+      <c r="J56" s="11" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="n"/>
@@ -1725,9 +1829,10 @@
         <v/>
       </c>
       <c r="F57" s="11" t="n"/>
-      <c r="G57" s="12" t="n"/>
+      <c r="G57" s="11" t="n"/>
       <c r="H57" s="12" t="n"/>
-      <c r="I57" s="11" t="n"/>
+      <c r="I57" s="12" t="n"/>
+      <c r="J57" s="11" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="n"/>
@@ -1742,9 +1847,10 @@
         <v/>
       </c>
       <c r="F58" s="11" t="n"/>
-      <c r="G58" s="12" t="n"/>
+      <c r="G58" s="11" t="n"/>
       <c r="H58" s="12" t="n"/>
-      <c r="I58" s="11" t="n"/>
+      <c r="I58" s="12" t="n"/>
+      <c r="J58" s="11" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="n"/>
@@ -1759,9 +1865,10 @@
         <v/>
       </c>
       <c r="F59" s="11" t="n"/>
-      <c r="G59" s="12" t="n"/>
+      <c r="G59" s="11" t="n"/>
       <c r="H59" s="12" t="n"/>
-      <c r="I59" s="11" t="n"/>
+      <c r="I59" s="12" t="n"/>
+      <c r="J59" s="11" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n"/>
@@ -1776,9 +1883,10 @@
         <v/>
       </c>
       <c r="F60" s="11" t="n"/>
-      <c r="G60" s="12" t="n"/>
+      <c r="G60" s="11" t="n"/>
       <c r="H60" s="12" t="n"/>
-      <c r="I60" s="11" t="n"/>
+      <c r="I60" s="12" t="n"/>
+      <c r="J60" s="11" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="n"/>
@@ -1793,12 +1901,18 @@
         <v/>
       </c>
       <c r="F61" s="11" t="n"/>
-      <c r="G61" s="12" t="n"/>
+      <c r="G61" s="11" t="n"/>
       <c r="H61" s="12" t="n"/>
-      <c r="I61" s="11" t="n"/>
+      <c r="I61" s="12" t="n"/>
+      <c r="J61" s="11" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I61"/>
+  <autoFilter ref="A1:J61"/>
+  <dataValidations count="1">
+    <dataValidation sqref="F2:F61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"유류비,정비비,기타"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1810,20 +1924,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1864,35 +1980,45 @@
       </c>
       <c r="E3" s="5" t="inlineStr">
         <is>
-          <t>차량유지비</t>
+          <t>유류비</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
+          <t>정비비</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>기타비용</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
           <t>하이패스</t>
         </is>
       </c>
-      <c r="G3" s="5" t="inlineStr">
+      <c r="I3" s="5" t="inlineStr">
         <is>
           <t>기사월급</t>
         </is>
       </c>
-      <c r="H3" s="5" t="inlineStr">
+      <c r="J3" s="5" t="inlineStr">
         <is>
           <t>차량보험</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="K3" s="5" t="inlineStr">
         <is>
           <t>총지출</t>
         </is>
       </c>
-      <c r="J3" s="5" t="inlineStr">
+      <c r="L3" s="5" t="inlineStr">
         <is>
           <t>순이익</t>
         </is>
       </c>
-      <c r="K3" s="5" t="inlineStr">
+      <c r="M3" s="5" t="inlineStr">
         <is>
           <t>이익률</t>
         </is>
@@ -1915,31 +2041,39 @@
         <v/>
       </c>
       <c r="E4" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A4,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A4+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A4,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A4+1,1))</f>
         <v/>
       </c>
       <c r="F4" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A4,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A4+1,1))</f>
+        <v/>
+      </c>
+      <c r="G4" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A4,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A4+1,1))</f>
+        <v/>
+      </c>
+      <c r="H4" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G4" s="15">
+      <c r="I4" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H4" s="15">
+      <c r="J4" s="15">
         <f>IF(A4=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I4" s="15">
-        <f>D4+E4+F4+G4+H4</f>
-        <v/>
-      </c>
-      <c r="J4" s="15">
-        <f>C4-I4</f>
-        <v/>
-      </c>
-      <c r="K4" s="16">
-        <f>IFERROR(J4/C4,0)</f>
+      <c r="K4" s="15">
+        <f>D4+E4+F4+G4+H4+I4+J4</f>
+        <v/>
+      </c>
+      <c r="L4" s="15">
+        <f>C4-K4</f>
+        <v/>
+      </c>
+      <c r="M4" s="16">
+        <f>IFERROR(L4/C4,0)</f>
         <v/>
       </c>
     </row>
@@ -1960,31 +2094,39 @@
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A5,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A5+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A5,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A5+1,1))</f>
         <v/>
       </c>
       <c r="F5" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A5,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A5+1,1))</f>
+        <v/>
+      </c>
+      <c r="G5" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A5,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A5+1,1))</f>
+        <v/>
+      </c>
+      <c r="H5" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G5" s="15">
+      <c r="I5" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H5" s="15">
+      <c r="J5" s="15">
         <f>IF(A5=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I5" s="15">
-        <f>D5+E5+F5+G5+H5</f>
-        <v/>
-      </c>
-      <c r="J5" s="15">
-        <f>C5-I5</f>
-        <v/>
-      </c>
-      <c r="K5" s="16">
-        <f>IFERROR(J5/C5,0)</f>
+      <c r="K5" s="15">
+        <f>D5+E5+F5+G5+H5+I5+J5</f>
+        <v/>
+      </c>
+      <c r="L5" s="15">
+        <f>C5-K5</f>
+        <v/>
+      </c>
+      <c r="M5" s="16">
+        <f>IFERROR(L5/C5,0)</f>
         <v/>
       </c>
     </row>
@@ -2005,31 +2147,39 @@
         <v/>
       </c>
       <c r="E6" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A6,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A6+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A6,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A6+1,1))</f>
         <v/>
       </c>
       <c r="F6" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A6,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A6+1,1))</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A6,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A6+1,1))</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G6" s="15">
+      <c r="I6" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H6" s="15">
+      <c r="J6" s="15">
         <f>IF(A6=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I6" s="15">
-        <f>D6+E6+F6+G6+H6</f>
-        <v/>
-      </c>
-      <c r="J6" s="15">
-        <f>C6-I6</f>
-        <v/>
-      </c>
-      <c r="K6" s="16">
-        <f>IFERROR(J6/C6,0)</f>
+      <c r="K6" s="15">
+        <f>D6+E6+F6+G6+H6+I6+J6</f>
+        <v/>
+      </c>
+      <c r="L6" s="15">
+        <f>C6-K6</f>
+        <v/>
+      </c>
+      <c r="M6" s="16">
+        <f>IFERROR(L6/C6,0)</f>
         <v/>
       </c>
     </row>
@@ -2050,31 +2200,39 @@
         <v/>
       </c>
       <c r="E7" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A7,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A7+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A7,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A7+1,1))</f>
         <v/>
       </c>
       <c r="F7" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A7,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A7+1,1))</f>
+        <v/>
+      </c>
+      <c r="G7" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A7,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A7+1,1))</f>
+        <v/>
+      </c>
+      <c r="H7" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G7" s="15">
+      <c r="I7" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H7" s="15">
+      <c r="J7" s="15">
         <f>IF(A7=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I7" s="15">
-        <f>D7+E7+F7+G7+H7</f>
-        <v/>
-      </c>
-      <c r="J7" s="15">
-        <f>C7-I7</f>
-        <v/>
-      </c>
-      <c r="K7" s="16">
-        <f>IFERROR(J7/C7,0)</f>
+      <c r="K7" s="15">
+        <f>D7+E7+F7+G7+H7+I7+J7</f>
+        <v/>
+      </c>
+      <c r="L7" s="15">
+        <f>C7-K7</f>
+        <v/>
+      </c>
+      <c r="M7" s="16">
+        <f>IFERROR(L7/C7,0)</f>
         <v/>
       </c>
     </row>
@@ -2095,31 +2253,39 @@
         <v/>
       </c>
       <c r="E8" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A8,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A8+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A8,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A8+1,1))</f>
         <v/>
       </c>
       <c r="F8" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A8,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A8+1,1))</f>
+        <v/>
+      </c>
+      <c r="G8" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A8,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A8+1,1))</f>
+        <v/>
+      </c>
+      <c r="H8" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G8" s="15">
+      <c r="I8" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H8" s="15">
+      <c r="J8" s="15">
         <f>IF(A8=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I8" s="15">
-        <f>D8+E8+F8+G8+H8</f>
-        <v/>
-      </c>
-      <c r="J8" s="15">
-        <f>C8-I8</f>
-        <v/>
-      </c>
-      <c r="K8" s="16">
-        <f>IFERROR(J8/C8,0)</f>
+      <c r="K8" s="15">
+        <f>D8+E8+F8+G8+H8+I8+J8</f>
+        <v/>
+      </c>
+      <c r="L8" s="15">
+        <f>C8-K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="16">
+        <f>IFERROR(L8/C8,0)</f>
         <v/>
       </c>
     </row>
@@ -2140,31 +2306,39 @@
         <v/>
       </c>
       <c r="E9" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A9,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A9+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A9,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A9+1,1))</f>
         <v/>
       </c>
       <c r="F9" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A9,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A9+1,1))</f>
+        <v/>
+      </c>
+      <c r="G9" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A9,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A9+1,1))</f>
+        <v/>
+      </c>
+      <c r="H9" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G9" s="15">
+      <c r="I9" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H9" s="15">
+      <c r="J9" s="15">
         <f>IF(A9=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I9" s="15">
-        <f>D9+E9+F9+G9+H9</f>
-        <v/>
-      </c>
-      <c r="J9" s="15">
-        <f>C9-I9</f>
-        <v/>
-      </c>
-      <c r="K9" s="16">
-        <f>IFERROR(J9/C9,0)</f>
+      <c r="K9" s="15">
+        <f>D9+E9+F9+G9+H9+I9+J9</f>
+        <v/>
+      </c>
+      <c r="L9" s="15">
+        <f>C9-K9</f>
+        <v/>
+      </c>
+      <c r="M9" s="16">
+        <f>IFERROR(L9/C9,0)</f>
         <v/>
       </c>
     </row>
@@ -2185,31 +2359,39 @@
         <v/>
       </c>
       <c r="E10" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A10,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A10+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A10,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A10+1,1))</f>
         <v/>
       </c>
       <c r="F10" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A10,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A10+1,1))</f>
+        <v/>
+      </c>
+      <c r="G10" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A10,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A10+1,1))</f>
+        <v/>
+      </c>
+      <c r="H10" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G10" s="15">
+      <c r="I10" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H10" s="15">
+      <c r="J10" s="15">
         <f>IF(A10=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I10" s="15">
-        <f>D10+E10+F10+G10+H10</f>
-        <v/>
-      </c>
-      <c r="J10" s="15">
-        <f>C10-I10</f>
-        <v/>
-      </c>
-      <c r="K10" s="16">
-        <f>IFERROR(J10/C10,0)</f>
+      <c r="K10" s="15">
+        <f>D10+E10+F10+G10+H10+I10+J10</f>
+        <v/>
+      </c>
+      <c r="L10" s="15">
+        <f>C10-K10</f>
+        <v/>
+      </c>
+      <c r="M10" s="16">
+        <f>IFERROR(L10/C10,0)</f>
         <v/>
       </c>
     </row>
@@ -2230,31 +2412,39 @@
         <v/>
       </c>
       <c r="E11" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A11,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A11+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A11,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A11+1,1))</f>
         <v/>
       </c>
       <c r="F11" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A11,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A11+1,1))</f>
+        <v/>
+      </c>
+      <c r="G11" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A11,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A11+1,1))</f>
+        <v/>
+      </c>
+      <c r="H11" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G11" s="15">
+      <c r="I11" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H11" s="15">
+      <c r="J11" s="15">
         <f>IF(A11=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I11" s="15">
-        <f>D11+E11+F11+G11+H11</f>
-        <v/>
-      </c>
-      <c r="J11" s="15">
-        <f>C11-I11</f>
-        <v/>
-      </c>
-      <c r="K11" s="16">
-        <f>IFERROR(J11/C11,0)</f>
+      <c r="K11" s="15">
+        <f>D11+E11+F11+G11+H11+I11+J11</f>
+        <v/>
+      </c>
+      <c r="L11" s="15">
+        <f>C11-K11</f>
+        <v/>
+      </c>
+      <c r="M11" s="16">
+        <f>IFERROR(L11/C11,0)</f>
         <v/>
       </c>
     </row>
@@ -2275,31 +2465,39 @@
         <v/>
       </c>
       <c r="E12" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A12,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A12+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A12,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A12+1,1))</f>
         <v/>
       </c>
       <c r="F12" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A12,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A12+1,1))</f>
+        <v/>
+      </c>
+      <c r="G12" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A12,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A12+1,1))</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G12" s="15">
+      <c r="I12" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H12" s="15">
+      <c r="J12" s="15">
         <f>IF(A12=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I12" s="15">
-        <f>D12+E12+F12+G12+H12</f>
-        <v/>
-      </c>
-      <c r="J12" s="15">
-        <f>C12-I12</f>
-        <v/>
-      </c>
-      <c r="K12" s="16">
-        <f>IFERROR(J12/C12,0)</f>
+      <c r="K12" s="15">
+        <f>D12+E12+F12+G12+H12+I12+J12</f>
+        <v/>
+      </c>
+      <c r="L12" s="15">
+        <f>C12-K12</f>
+        <v/>
+      </c>
+      <c r="M12" s="16">
+        <f>IFERROR(L12/C12,0)</f>
         <v/>
       </c>
     </row>
@@ -2320,31 +2518,39 @@
         <v/>
       </c>
       <c r="E13" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A13,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A13+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A13,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A13+1,1))</f>
         <v/>
       </c>
       <c r="F13" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A13,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A13+1,1))</f>
+        <v/>
+      </c>
+      <c r="G13" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A13,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A13+1,1))</f>
+        <v/>
+      </c>
+      <c r="H13" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G13" s="15">
+      <c r="I13" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H13" s="15">
+      <c r="J13" s="15">
         <f>IF(A13=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I13" s="15">
-        <f>D13+E13+F13+G13+H13</f>
-        <v/>
-      </c>
-      <c r="J13" s="15">
-        <f>C13-I13</f>
-        <v/>
-      </c>
-      <c r="K13" s="16">
-        <f>IFERROR(J13/C13,0)</f>
+      <c r="K13" s="15">
+        <f>D13+E13+F13+G13+H13+I13+J13</f>
+        <v/>
+      </c>
+      <c r="L13" s="15">
+        <f>C13-K13</f>
+        <v/>
+      </c>
+      <c r="M13" s="16">
+        <f>IFERROR(L13/C13,0)</f>
         <v/>
       </c>
     </row>
@@ -2365,31 +2571,39 @@
         <v/>
       </c>
       <c r="E14" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A14,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A14+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A14,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A14+1,1))</f>
         <v/>
       </c>
       <c r="F14" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A14,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A14+1,1))</f>
+        <v/>
+      </c>
+      <c r="G14" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A14,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A14+1,1))</f>
+        <v/>
+      </c>
+      <c r="H14" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G14" s="15">
+      <c r="I14" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H14" s="15">
+      <c r="J14" s="15">
         <f>IF(A14=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I14" s="15">
-        <f>D14+E14+F14+G14+H14</f>
-        <v/>
-      </c>
-      <c r="J14" s="15">
-        <f>C14-I14</f>
-        <v/>
-      </c>
-      <c r="K14" s="16">
-        <f>IFERROR(J14/C14,0)</f>
+      <c r="K14" s="15">
+        <f>D14+E14+F14+G14+H14+I14+J14</f>
+        <v/>
+      </c>
+      <c r="L14" s="15">
+        <f>C14-K14</f>
+        <v/>
+      </c>
+      <c r="M14" s="16">
+        <f>IFERROR(L14/C14,0)</f>
         <v/>
       </c>
     </row>
@@ -2410,31 +2624,39 @@
         <v/>
       </c>
       <c r="E15" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A15,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A15+1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A15,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A15+1,1))</f>
         <v/>
       </c>
       <c r="F15" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A15,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A15+1,1))</f>
+        <v/>
+      </c>
+      <c r="G15" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($B$1,A15,1),일일기록!$A:$A,"&lt;"&amp;DATE($B$1,A15+1,1))</f>
+        <v/>
+      </c>
+      <c r="H15" s="15">
         <f>고정비설정!$B$5</f>
         <v/>
       </c>
-      <c r="G15" s="15">
+      <c r="I15" s="15">
         <f>고정비설정!$B$4</f>
         <v/>
       </c>
-      <c r="H15" s="15">
+      <c r="J15" s="15">
         <f>IF(A15=고정비설정!$B$7,고정비설정!$B$6,0)</f>
         <v/>
       </c>
-      <c r="I15" s="15">
-        <f>D15+E15+F15+G15+H15</f>
-        <v/>
-      </c>
-      <c r="J15" s="15">
-        <f>C15-I15</f>
-        <v/>
-      </c>
-      <c r="K15" s="16">
-        <f>IFERROR(J15/C15,0)</f>
+      <c r="K15" s="15">
+        <f>D15+E15+F15+G15+H15+I15+J15</f>
+        <v/>
+      </c>
+      <c r="L15" s="15">
+        <f>C15-K15</f>
+        <v/>
+      </c>
+      <c r="M15" s="16">
+        <f>IFERROR(L15/C15,0)</f>
         <v/>
       </c>
     </row>
@@ -2477,8 +2699,16 @@
         <f>SUM(J4:J15)</f>
         <v/>
       </c>
-      <c r="K16" s="20">
-        <f>IFERROR(J16/C16,0)</f>
+      <c r="K16" s="19">
+        <f>SUM(K4:K15)</f>
+        <v/>
+      </c>
+      <c r="L16" s="19">
+        <f>SUM(L4:L15)</f>
+        <v/>
+      </c>
+      <c r="M16" s="20">
+        <f>IFERROR(L16/C16,0)</f>
         <v/>
       </c>
     </row>
@@ -2496,20 +2726,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2535,35 +2767,45 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>차량유지비</t>
+          <t>유류비</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
+          <t>정비비</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
+          <t>기타비용</t>
+        </is>
+      </c>
+      <c r="H1" s="5" t="inlineStr">
+        <is>
           <t>하이패스(연)</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>기사월급(연)</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>차량보험</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>총지출</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>순이익</t>
         </is>
       </c>
-      <c r="K1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
         <is>
           <t>수익률</t>
         </is>
@@ -2586,31 +2828,39 @@
         <v/>
       </c>
       <c r="E2" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($A2,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A2+1,1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($A2,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A2+1,1,1))</f>
         <v/>
       </c>
       <c r="F2" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($A2,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A2+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="G2" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($A2,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A2+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="H2" s="15">
         <f>고정비설정!$B$5*12</f>
         <v/>
       </c>
-      <c r="G2" s="15">
+      <c r="I2" s="15">
         <f>고정비설정!$B$4*12</f>
         <v/>
       </c>
-      <c r="H2" s="15">
+      <c r="J2" s="15">
         <f>고정비설정!$B$6</f>
         <v/>
       </c>
-      <c r="I2" s="15">
-        <f>D2+E2+F2+G2+H2</f>
-        <v/>
-      </c>
-      <c r="J2" s="15">
-        <f>C2-I2</f>
-        <v/>
-      </c>
-      <c r="K2" s="16">
-        <f>IFERROR(J2/C2,0)</f>
+      <c r="K2" s="15">
+        <f>D2+E2+F2+G2+H2+I2+J2</f>
+        <v/>
+      </c>
+      <c r="L2" s="15">
+        <f>C2-K2</f>
+        <v/>
+      </c>
+      <c r="M2" s="16">
+        <f>IFERROR(L2/C2,0)</f>
         <v/>
       </c>
     </row>
@@ -2631,31 +2881,39 @@
         <v/>
       </c>
       <c r="E3" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($A3,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A3+1,1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($A3,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A3+1,1,1))</f>
         <v/>
       </c>
       <c r="F3" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($A3,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A3+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="G3" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($A3,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A3+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="H3" s="15">
         <f>고정비설정!$B$5*12</f>
         <v/>
       </c>
-      <c r="G3" s="15">
+      <c r="I3" s="15">
         <f>고정비설정!$B$4*12</f>
         <v/>
       </c>
-      <c r="H3" s="15">
+      <c r="J3" s="15">
         <f>고정비설정!$B$6</f>
         <v/>
       </c>
-      <c r="I3" s="15">
-        <f>D3+E3+F3+G3+H3</f>
-        <v/>
-      </c>
-      <c r="J3" s="15">
-        <f>C3-I3</f>
-        <v/>
-      </c>
-      <c r="K3" s="16">
-        <f>IFERROR(J3/C3,0)</f>
+      <c r="K3" s="15">
+        <f>D3+E3+F3+G3+H3+I3+J3</f>
+        <v/>
+      </c>
+      <c r="L3" s="15">
+        <f>C3-K3</f>
+        <v/>
+      </c>
+      <c r="M3" s="16">
+        <f>IFERROR(L3/C3,0)</f>
         <v/>
       </c>
     </row>
@@ -2676,31 +2934,39 @@
         <v/>
       </c>
       <c r="E4" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($A4,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A4+1,1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($A4,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A4+1,1,1))</f>
         <v/>
       </c>
       <c r="F4" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($A4,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A4+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="G4" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($A4,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A4+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="H4" s="15">
         <f>고정비설정!$B$5*12</f>
         <v/>
       </c>
-      <c r="G4" s="15">
+      <c r="I4" s="15">
         <f>고정비설정!$B$4*12</f>
         <v/>
       </c>
-      <c r="H4" s="15">
+      <c r="J4" s="15">
         <f>고정비설정!$B$6</f>
         <v/>
       </c>
-      <c r="I4" s="15">
-        <f>D4+E4+F4+G4+H4</f>
-        <v/>
-      </c>
-      <c r="J4" s="15">
-        <f>C4-I4</f>
-        <v/>
-      </c>
-      <c r="K4" s="16">
-        <f>IFERROR(J4/C4,0)</f>
+      <c r="K4" s="15">
+        <f>D4+E4+F4+G4+H4+I4+J4</f>
+        <v/>
+      </c>
+      <c r="L4" s="15">
+        <f>C4-K4</f>
+        <v/>
+      </c>
+      <c r="M4" s="16">
+        <f>IFERROR(L4/C4,0)</f>
         <v/>
       </c>
     </row>
@@ -2721,31 +2987,39 @@
         <v/>
       </c>
       <c r="E5" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($A5,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A5+1,1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($A5,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A5+1,1,1))</f>
         <v/>
       </c>
       <c r="F5" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($A5,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A5+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="G5" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($A5,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A5+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="H5" s="15">
         <f>고정비설정!$B$5*12</f>
         <v/>
       </c>
-      <c r="G5" s="15">
+      <c r="I5" s="15">
         <f>고정비설정!$B$4*12</f>
         <v/>
       </c>
-      <c r="H5" s="15">
+      <c r="J5" s="15">
         <f>고정비설정!$B$6</f>
         <v/>
       </c>
-      <c r="I5" s="15">
-        <f>D5+E5+F5+G5+H5</f>
-        <v/>
-      </c>
-      <c r="J5" s="15">
-        <f>C5-I5</f>
-        <v/>
-      </c>
-      <c r="K5" s="16">
-        <f>IFERROR(J5/C5,0)</f>
+      <c r="K5" s="15">
+        <f>D5+E5+F5+G5+H5+I5+J5</f>
+        <v/>
+      </c>
+      <c r="L5" s="15">
+        <f>C5-K5</f>
+        <v/>
+      </c>
+      <c r="M5" s="16">
+        <f>IFERROR(L5/C5,0)</f>
         <v/>
       </c>
     </row>
@@ -2766,31 +3040,39 @@
         <v/>
       </c>
       <c r="E6" s="15">
-        <f>SUMIFS(일일기록!$G:$G,일일기록!$A:$A,"&gt;="&amp;DATE($A6,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A6+1,1,1))</f>
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"유류비",일일기록!$A:$A,"&gt;="&amp;DATE($A6,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A6+1,1,1))</f>
         <v/>
       </c>
       <c r="F6" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"정비비",일일기록!$A:$A,"&gt;="&amp;DATE($A6,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A6+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="G6" s="15">
+        <f>SUMIFS(일일기록!$H:$H,일일기록!$F:$F,"기타",일일기록!$A:$A,"&gt;="&amp;DATE($A6,1,1),일일기록!$A:$A,"&lt;"&amp;DATE($A6+1,1,1))</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
         <f>고정비설정!$B$5*12</f>
         <v/>
       </c>
-      <c r="G6" s="15">
+      <c r="I6" s="15">
         <f>고정비설정!$B$4*12</f>
         <v/>
       </c>
-      <c r="H6" s="15">
+      <c r="J6" s="15">
         <f>고정비설정!$B$6</f>
         <v/>
       </c>
-      <c r="I6" s="15">
-        <f>D6+E6+F6+G6+H6</f>
-        <v/>
-      </c>
-      <c r="J6" s="15">
-        <f>C6-I6</f>
-        <v/>
-      </c>
-      <c r="K6" s="16">
-        <f>IFERROR(J6/C6,0)</f>
+      <c r="K6" s="15">
+        <f>D6+E6+F6+G6+H6+I6+J6</f>
+        <v/>
+      </c>
+      <c r="L6" s="15">
+        <f>C6-K6</f>
+        <v/>
+      </c>
+      <c r="M6" s="16">
+        <f>IFERROR(L6/C6,0)</f>
         <v/>
       </c>
     </row>
@@ -2805,7 +3087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2833,14 +3115,14 @@
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="22" t="inlineStr">
         <is>
-          <t>- ① '고정비설정' 시트: 단가(원/판), 기사월급, 하이패스, 차량보험료 등 거의 안 바뀌는 값을 한 번만 입력해두세요. 나중에 값이 바뀌면 여기만 수정하면 전체에 반영됩니다.</t>
+          <t>- ① '고정비설정' 시트: 단가(원/판), 기사월급, 하이패스, 차량보험료 등 거의 안 바뀌는 값을 한 번만 입력해두세요.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="22" t="inlineStr">
         <is>
-          <t>- ② '일일기록' 시트: 매일 운행/정비 후 날짜·농장·판수 또는 차량유지내용/비용·하이패스만 입력하면 단가·매출액은 자동 계산됩니다.</t>
+          <t>- ② '일일기록' 시트: 매일 운행/정비 후 날짜·농장·판수 또는 지출구분/지출내용/지출금액·하이패스만 입력하면 단가·매출액은 자동 계산됩니다.</t>
         </is>
       </c>
     </row>
@@ -2854,21 +3136,21 @@
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="22" t="inlineStr">
         <is>
-          <t>-    - 정비/유류/톨게이트 등 지출 건: 같은 날짜 행에 차량유지내용/차량유지비용 또는 하이패스만 입력</t>
+          <t>-    - 지출 건(유류/정비/기타): 지출구분(드롭다운에서 유류비/정비비/기타 선택) + 지출내용(메모) + 지출금액 입력</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="22" t="inlineStr">
         <is>
-          <t>-    - 특정 달의 정비내역만 보고 싶으면 '일일기록' 시트 헤더의 필터 버튼으로 날짜(월) + 차량유지내용을 필터링하세요 (자동 필터 적용됨).</t>
+          <t>-    - 특정 달의 정비내역만 보고 싶으면 헤더의 필터 버튼으로 날짜(월) + 지출구분을 필터링하세요.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="22" t="inlineStr">
         <is>
-          <t>- ③ '월별손익' 시트: 상단 노란색 '기준연도' 셀(B1)만 바꾸면 1~12월 매출/지출/순이익/이익률이 자동 집계됩니다.</t>
+          <t>- ③ '월별손익' 시트: 상단 노란색 '기준연도' 셀(B1)만 바꾸면 1~12월 매출·부가세·유류비·정비비·기타비용·순이익·이익률이 자동 집계됩니다.</t>
         </is>
       </c>
     </row>
@@ -2900,19 +3182,11 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t>- 이 파일은 참고로 제공된 기존 관리 파일(1월~12월/과년/년간총액 구조)의 항목을 그대로 반영하되, 월간·연간 합계를 손으로 다시 옮겨 적지 않아도 되도록 수식으로 자동 연결한 버전입니다.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="12">
     <mergeCell ref="A11:F11"/>
     <mergeCell ref="A10:F10"/>
     <mergeCell ref="A13:F13"/>
-    <mergeCell ref="A14:F14"/>
     <mergeCell ref="A5:F5"/>
     <mergeCell ref="A9:F9"/>
     <mergeCell ref="A8:F8"/>

</xml_diff>